<commit_message>
20260613_01_kfold_deberta_default_OOF_F1_0.9127, 20260613_02_kfold_deberta_thresh0.57_OOF_F1_0.9144, 20260613_03_roberta_F1_0.8929, 20260613_04_deberta_v3_F1_0.9098, 20260611_02_ensemble_tf_idf_logreg_deberta_v3_F1_0.9242
</commit_message>
<xml_diff>
--- a/Experiments_NLP.xlsx
+++ b/Experiments_NLP.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://smu-my.sharepoint.com/personal/kh_nguyen_2025_mitb_smu_edu_sg/Documents/Data_Science/SMU/Study/Term 2/CS605 NLP for Smart Assistants/Assignment/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="34" documentId="8_{CB199A4B-7D07-4B0C-BB92-4FC6BF07BB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C6DD3FA6-2882-489C-9D99-9E62BE0C318A}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="8_{CB199A4B-7D07-4B0C-BB92-4FC6BF07BB6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06CB467E-CA4B-4C98-A87A-1E585C7937CF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{553DC2F9-6C9A-46BB-ABFD-28C82DBA10AE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
   <si>
     <t>20260611_04_deberta_v3_F1_0.9214</t>
   </si>
@@ -96,6 +96,16 @@
   </si>
   <si>
     <t>Note</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>weight = 0.5 if 0.3 &lt;= quality_score &lt; 0.5 else 1.0</t>
+  </si>
+  <si>
+    <t>Run Claude: 26min
+Run Groq: 5 hours</t>
   </si>
 </sst>
 </file>
@@ -134,9 +144,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -152,6 +165,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>212593</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>172899</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0EDDA5B1-F47C-37E7-BC59-8045256F6E89}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="3840480"/>
+          <a:ext cx="6133333" cy="3647619"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -471,154 +533,197 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{22CC1786-9B20-4260-A956-5D6B7C779879}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="62.21875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="50.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
     <col min="3" max="3" width="10.77734375" customWidth="1"/>
+    <col min="4" max="4" width="62.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D1" t="s">
         <v>8</v>
       </c>
-      <c r="B1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>2</v>
+      </c>
+      <c r="B2">
+        <v>0.81081000000000003</v>
+      </c>
+      <c r="D2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C2">
-        <v>0.81081000000000003</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3">
+        <v>0.81281000000000003</v>
+      </c>
+      <c r="D3" t="s">
         <v>9</v>
       </c>
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0.81281000000000003</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>0.80066000000000004</v>
+      </c>
+      <c r="D4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>0.80066000000000004</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E4" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5">
+        <v>0.76112000000000002</v>
+      </c>
+      <c r="D5" t="s">
         <v>9</v>
       </c>
-      <c r="B5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C5">
-        <v>0.76112000000000002</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1">
+        <v>0.81299999999999994</v>
+      </c>
+      <c r="D6" t="s">
         <v>9</v>
       </c>
-      <c r="B6" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" s="1">
-        <v>0.81299999999999994</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7">
+        <v>0.81238999999999995</v>
+      </c>
+      <c r="D7" t="s">
         <v>9</v>
       </c>
-      <c r="B7" t="s">
-        <v>7</v>
-      </c>
-      <c r="C7">
-        <v>0.81238999999999995</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8">
+        <v>0.82538999999999996</v>
+      </c>
+      <c r="D8" t="s">
         <v>12</v>
       </c>
-      <c r="B8" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8">
-        <v>0.82538999999999996</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E8" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9">
+        <v>0.82147999999999999</v>
+      </c>
+      <c r="D9" t="s">
         <v>12</v>
       </c>
-      <c r="B9" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9">
-        <v>0.82147999999999999</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10">
+        <v>0.82669999999999999</v>
+      </c>
+      <c r="D10" t="s">
         <v>14</v>
       </c>
-      <c r="B10" t="s">
-        <v>13</v>
-      </c>
-      <c r="C10">
-        <v>0.82669999999999999</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E10" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11">
+        <v>0.82801999999999998</v>
+      </c>
+      <c r="C11" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" t="s">
         <v>14</v>
       </c>
-      <c r="B11" t="s">
-        <v>15</v>
-      </c>
-      <c r="C11">
-        <v>0.82801999999999998</v>
-      </c>
-      <c r="D11" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="E11" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12">
+        <v>0.82747000000000004</v>
+      </c>
+      <c r="D12" t="s">
         <v>14</v>
       </c>
-      <c r="B12" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12">
-        <v>0.82747000000000004</v>
+      <c r="E12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="57.6" x14ac:dyDescent="0.3">
+      <c r="C13" s="2" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>